<commit_message>
Updated to add to the technical guide menu/ a button to the intro page for the admin data guide
</commit_message>
<xml_diff>
--- a/administrative-database-guidance/data/tbl_ucas_MIOM_outcomes.xlsx
+++ b/administrative-database-guidance/data/tbl_ucas_MIOM_outcomes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikaylaBoginsky\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikaylaBoginsky\Documents\technicalguide\administrative-database-guidance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{750871AC-45EA-468A-8F0D-01423CAEAB91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E6470C-EC1C-44F6-B8B6-3092971678FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4350" yWindow="1350" windowWidth="14400" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Edited to change mention of Strobe to Outreach Evaluator.
</commit_message>
<xml_diff>
--- a/administrative-database-guidance/data/tbl_ucas_MIOM_outcomes.xlsx
+++ b/administrative-database-guidance/data/tbl_ucas_MIOM_outcomes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikaylaBoginsky\Documents\technicalguide\administrative-database-guidance\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robsummers.AzureAD\Documents\R\technicalguide\administrative-database-guidance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321BB416-134F-41FC-B81C-3D529B88AB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6708596-95D4-4880-9F87-00B57F735AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="4875" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
   <si>
-    <t>Outcome measure *</t>
-  </si>
-  <si>
     <t>Data to be collected</t>
   </si>
   <si>
@@ -50,9 +47,6 @@
   </si>
   <si>
     <t>Individual data collected by UCAS in February before university entry. Data available to access in the October of the year of entry</t>
-  </si>
-  <si>
-    <t>UCAS strobe</t>
   </si>
   <si>
     <t>Exploratory: Number of offers (zero to five)</t>
@@ -82,6 +76,12 @@
   <si>
     <t xml:space="preserve">Spring of the academic year they begin (April 2024 and 2025)
 </t>
+  </si>
+  <si>
+    <t>UCAS Outreach Evaluator</t>
+  </si>
+  <si>
+    <t>Outcome measure</t>
   </si>
 </sst>
 </file>
@@ -365,91 +365,91 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="B2:F6"/>
-  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:6" ht="29.5" x14ac:dyDescent="0.7">
+    <row r="2" spans="2:6" ht="30" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+    </row>
+    <row r="3" spans="2:6" ht="270" x14ac:dyDescent="0.35">
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="255" x14ac:dyDescent="0.95">
-      <c r="B3" s="3" t="s">
+    <row r="4" spans="2:6" ht="144" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F4" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" ht="234" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="4" spans="2:6" ht="136" x14ac:dyDescent="0.95">
-      <c r="B4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" ht="221" x14ac:dyDescent="0.95">
-      <c r="B5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="4" t="s">
+    <row r="6" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.95">
-      <c r="B6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>